<commit_message>
Correct U-values of non-residential partially retrofitted buildings Correct outer wall areas of terraced houses.
</commit_message>
<xml_diff>
--- a/districtgenerator/data/SIA2024.xlsx
+++ b/districtgenerator/data/SIA2024.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PycharmProjects\districtgenerator\districtgenerator\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C46E1CC7-33C6-408B-814C-84B809AB8B07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DA02AE6-9A84-4653-AE85-1DECD4D79550}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="16440" windowHeight="28320" tabRatio="799" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11835" yWindow="-16335" windowWidth="29040" windowHeight="15720" tabRatio="799" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SIA2024" sheetId="13" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="210">
   <si>
     <t>°C</t>
   </si>
@@ -657,6 +657,12 @@
   </si>
   <si>
     <t>store</t>
+  </si>
+  <si>
+    <t>Beheizte Zone</t>
+  </si>
+  <si>
+    <t>Anteil beheizter Fläche</t>
   </si>
 </sst>
 </file>
@@ -1208,7 +1214,7 @@
       <protection hidden="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
@@ -1272,6 +1278,12 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="29" xfId="18" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="18" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="18" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1586,40 +1598,40 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:CU48"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:DC48"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="39.7109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.28515625" customWidth="1"/>
-    <col min="6" max="6" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.85546875" customWidth="1"/>
-    <col min="9" max="10" width="13.85546875" customWidth="1"/>
-    <col min="11" max="11" width="28.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="26.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="24.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="19.140625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="24.5703125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.140625" customWidth="1"/>
-    <col min="86" max="86" width="22.7109375" bestFit="1" customWidth="1"/>
-    <col min="87" max="87" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="88" max="90" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="39.6640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.33203125" customWidth="1"/>
+    <col min="6" max="6" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.88671875" customWidth="1"/>
+    <col min="9" max="10" width="13.88671875" customWidth="1"/>
+    <col min="11" max="11" width="28.5546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="26.33203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="24.44140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="19.109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="24.5546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.109375" customWidth="1"/>
+    <col min="86" max="86" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="87" max="87" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="88" max="90" width="6.44140625" bestFit="1" customWidth="1"/>
     <col min="91" max="91" width="22" bestFit="1" customWidth="1"/>
-    <col min="92" max="92" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="92" max="92" width="6.44140625" bestFit="1" customWidth="1"/>
     <col min="93" max="93" width="9" bestFit="1" customWidth="1"/>
-    <col min="94" max="94" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="95" max="95" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="96" max="96" width="7.140625" bestFit="1" customWidth="1"/>
-    <col min="97" max="97" width="6.140625" bestFit="1" customWidth="1"/>
-    <col min="98" max="98" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="94" max="94" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="95" max="95" width="7.88671875" bestFit="1" customWidth="1"/>
+    <col min="96" max="96" width="7.109375" bestFit="1" customWidth="1"/>
+    <col min="97" max="97" width="6.109375" bestFit="1" customWidth="1"/>
+    <col min="98" max="98" width="9.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:99" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:107" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="23"/>
       <c r="B1" s="27"/>
       <c r="C1" s="23" t="s">
@@ -1742,8 +1754,14 @@
       <c r="CH1" s="5" t="s">
         <v>188</v>
       </c>
+      <c r="CY1" s="59" t="s">
+        <v>209</v>
+      </c>
+      <c r="CZ1" s="59"/>
+      <c r="DA1" s="59"/>
+      <c r="DB1" s="59"/>
     </row>
-    <row r="2" spans="1:99" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:107" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="44" t="s">
         <v>65</v>
       </c>
@@ -2038,8 +2056,23 @@
       <c r="CT2" s="4" t="s">
         <v>196</v>
       </c>
+      <c r="CY2" t="s">
+        <v>208</v>
+      </c>
+      <c r="CZ2" t="s">
+        <v>203</v>
+      </c>
+      <c r="DA2" t="s">
+        <v>205</v>
+      </c>
+      <c r="DB2" t="s">
+        <v>204</v>
+      </c>
+      <c r="DC2" t="s">
+        <v>206</v>
+      </c>
     </row>
-    <row r="3" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A3" s="28" t="s">
         <v>144</v>
       </c>
@@ -2326,8 +2359,28 @@
         <f t="shared" ref="CU3:CU47" si="0">CJ3*Q3+CJ3*S3</f>
         <v>0</v>
       </c>
+      <c r="CY3">
+        <f>IF(D3&gt;=19,1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="CZ3">
+        <f>CY3*CJ3</f>
+        <v>0</v>
+      </c>
+      <c r="DA3">
+        <f>CY3*CK3</f>
+        <v>0</v>
+      </c>
+      <c r="DB3">
+        <f>CY3*CL3</f>
+        <v>0</v>
+      </c>
+      <c r="DC3">
+        <f>CY3*CM3</f>
+        <v>0</v>
+      </c>
     </row>
-    <row r="4" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>145</v>
       </c>
@@ -2614,8 +2667,28 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="CY4">
+        <f t="shared" ref="CY4:CY47" si="1">IF(D4&gt;=19,1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="CZ4">
+        <f t="shared" ref="CZ4:CZ47" si="2">CY4*CJ4</f>
+        <v>0</v>
+      </c>
+      <c r="DA4">
+        <f t="shared" ref="DA4:DA47" si="3">CY4*CK4</f>
+        <v>0</v>
+      </c>
+      <c r="DB4">
+        <f t="shared" ref="DB4:DB47" si="4">CY4*CL4</f>
+        <v>0</v>
+      </c>
+      <c r="DC4">
+        <f t="shared" ref="DC4:DC47" si="5">CY4*CM4</f>
+        <v>0</v>
+      </c>
     </row>
-    <row r="5" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>146</v>
       </c>
@@ -2902,8 +2975,28 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="CY5">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="CZ5">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DA5">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="DB5">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC5">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="6" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>147</v>
       </c>
@@ -3190,8 +3283,28 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="CY6">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="CZ6">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DA6">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="DB6">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC6">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="7" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
         <v>148</v>
       </c>
@@ -3488,8 +3601,28 @@
         <f t="shared" si="0"/>
         <v>1.73</v>
       </c>
+      <c r="CY7">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="CZ7">
+        <f t="shared" si="2"/>
+        <v>0.1</v>
+      </c>
+      <c r="DA7">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="DB7">
+        <f t="shared" si="4"/>
+        <v>0.05</v>
+      </c>
+      <c r="DC7">
+        <f t="shared" si="5"/>
+        <v>0.05</v>
+      </c>
     </row>
-    <row r="8" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
         <v>149</v>
       </c>
@@ -3776,8 +3909,28 @@
         <f t="shared" si="0"/>
         <v>12.3</v>
       </c>
+      <c r="CY8">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="CZ8">
+        <f t="shared" si="2"/>
+        <v>0.5</v>
+      </c>
+      <c r="DA8">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="DB8">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC8">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="9" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="s">
         <v>150</v>
       </c>
@@ -4064,8 +4217,28 @@
         <f t="shared" si="0"/>
         <v>0.8899999999999999</v>
       </c>
+      <c r="CY9">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="CZ9">
+        <f t="shared" si="2"/>
+        <v>0.1</v>
+      </c>
+      <c r="DA9">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="DB9">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC9">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="10" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
         <v>151</v>
       </c>
@@ -4352,8 +4525,28 @@
         <f t="shared" si="0"/>
         <v>0.57000000000000006</v>
       </c>
+      <c r="CY10">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="CZ10">
+        <f t="shared" si="2"/>
+        <v>0.05</v>
+      </c>
+      <c r="DA10">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="DB10">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC10">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="11" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
         <v>152</v>
       </c>
@@ -4640,8 +4833,28 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="CY11">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="CZ11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DA11">
+        <f t="shared" si="3"/>
+        <v>0.5</v>
+      </c>
+      <c r="DB11">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC11">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="12" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A12" s="9" t="s">
         <v>153</v>
       </c>
@@ -4928,8 +5141,28 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="CY12">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="CZ12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DA12">
+        <f t="shared" si="3"/>
+        <v>0.05</v>
+      </c>
+      <c r="DB12">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC12">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="13" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A13" s="9" t="s">
         <v>154</v>
       </c>
@@ -5216,8 +5449,28 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="CY13">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="CZ13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DA13">
+        <f t="shared" si="3"/>
+        <v>0.05</v>
+      </c>
+      <c r="DB13">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC13">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="14" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A14" s="9" t="s">
         <v>155</v>
       </c>
@@ -5504,8 +5757,28 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="CY14">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="CZ14">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DA14">
+        <f t="shared" si="3"/>
+        <v>0.05</v>
+      </c>
+      <c r="DB14">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC14">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="15" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A15" s="9" t="s">
         <v>156</v>
       </c>
@@ -5792,8 +6065,28 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="CY15">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="CZ15">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DA15">
+        <f t="shared" si="3"/>
+        <v>0.05</v>
+      </c>
+      <c r="DB15">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC15">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="16" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A16" s="9" t="s">
         <v>157</v>
       </c>
@@ -6081,8 +6374,28 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="CY16">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="CZ16">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DA16">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="DB16">
+        <f t="shared" si="4"/>
+        <v>0.64999999999999991</v>
+      </c>
+      <c r="DC16">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="17" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A17" s="9" t="s">
         <v>158</v>
       </c>
@@ -6369,8 +6682,28 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="CY17">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="CZ17">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DA17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="DB17">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC17">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="18" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A18" s="9" t="s">
         <v>159</v>
       </c>
@@ -6657,8 +6990,28 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="CY18">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="CZ18">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DA18">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="DB18">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC18">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="19" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A19" s="9" t="s">
         <v>160</v>
       </c>
@@ -6945,8 +7298,28 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="CY19">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="CZ19">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DA19">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="DB19">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC19">
+        <f t="shared" si="5"/>
+        <v>0.6</v>
+      </c>
     </row>
-    <row r="20" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A20" s="9" t="s">
         <v>161</v>
       </c>
@@ -7233,8 +7606,28 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="CY20">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="CZ20">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DA20">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="DB20">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC20">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="21" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A21" s="9" t="s">
         <v>162</v>
       </c>
@@ -7521,8 +7914,28 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="CY21">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="CZ21">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DA21">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="DB21">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC21">
+        <f t="shared" si="5"/>
+        <v>0.1</v>
+      </c>
     </row>
-    <row r="22" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A22" s="9" t="s">
         <v>163</v>
       </c>
@@ -7809,8 +8222,28 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="CY22">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="CZ22">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DA22">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="DB22">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC22">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="23" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A23" s="9" t="s">
         <v>164</v>
       </c>
@@ -8099,8 +8532,28 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="CY23">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="CZ23">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DA23">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="DB23">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC23">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="24" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A24" s="9" t="s">
         <v>165</v>
       </c>
@@ -8389,8 +8842,28 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="CY24">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="CZ24">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DA24">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="DB24">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC24">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="25" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A25" s="9" t="s">
         <v>166</v>
       </c>
@@ -8679,8 +9152,28 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="CY25">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="CZ25">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DA25">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="DB25">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC25">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="26" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A26" s="9" t="s">
         <v>167</v>
       </c>
@@ -8969,8 +9462,28 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="CY26">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="CZ26">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DA26">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="DB26">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC26">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="27" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A27" s="9" t="s">
         <v>168</v>
       </c>
@@ -9259,8 +9772,28 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="CY27">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="CZ27">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DA27">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="DB27">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC27">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="28" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A28" s="9" t="s">
         <v>169</v>
       </c>
@@ -9549,8 +10082,28 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="CY28">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="CZ28">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DA28">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="DB28">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC28">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="29" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A29" s="9" t="s">
         <v>170</v>
       </c>
@@ -9839,8 +10392,28 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="CY29">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="CZ29">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DA29">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="DB29">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC29">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="30" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A30" s="9" t="s">
         <v>171</v>
       </c>
@@ -10129,8 +10702,28 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="CY30">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="CZ30">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DA30">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="DB30">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC30">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="31" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A31" s="9" t="s">
         <v>172</v>
       </c>
@@ -10417,8 +11010,28 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="CY31">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="CZ31">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DA31">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="DB31">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC31">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="32" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A32" s="9" t="s">
         <v>173</v>
       </c>
@@ -10707,8 +11320,28 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="CY32">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="CZ32">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DA32">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="DB32">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC32">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="33" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A33" s="9" t="s">
         <v>174</v>
       </c>
@@ -10997,8 +11630,28 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="CY33">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="CZ33">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DA33">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="DB33">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC33">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="34" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A34" s="9" t="s">
         <v>175</v>
       </c>
@@ -11285,8 +11938,28 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="CY34">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="CZ34">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DA34">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="DB34">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC34">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="35" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A35" s="9" t="s">
         <v>176</v>
       </c>
@@ -11575,8 +12248,28 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="CY35">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="CZ35">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DA35">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="DB35">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC35">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="36" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A36" s="9" t="s">
         <v>177</v>
       </c>
@@ -11875,8 +12568,28 @@
         <f t="shared" si="0"/>
         <v>0.34</v>
       </c>
+      <c r="CY36">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="CZ36">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DA36">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="DB36">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC36">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="37" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A37" s="9" t="s">
         <v>178</v>
       </c>
@@ -12167,8 +12880,28 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="CY37">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="CZ37">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DA37">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="DB37">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC37">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="38" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A38" s="9" t="s">
         <v>179</v>
       </c>
@@ -12459,8 +13192,28 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="CY38">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="CZ38">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DA38">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="DB38">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC38">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="39" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A39" s="9" t="s">
         <v>180</v>
       </c>
@@ -12759,8 +13512,28 @@
         <f t="shared" si="0"/>
         <v>2.0000000000000004E-2</v>
       </c>
+      <c r="CY39">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="CZ39">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DA39">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="DB39">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC39">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="40" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A40" s="9" t="s">
         <v>181</v>
       </c>
@@ -13047,8 +13820,28 @@
         <f t="shared" si="0"/>
         <v>1.37</v>
       </c>
+      <c r="CY40">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="CZ40">
+        <f t="shared" si="2"/>
+        <v>0.02</v>
+      </c>
+      <c r="DA40">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="DB40">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC40">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="41" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A41" s="9" t="s">
         <v>182</v>
       </c>
@@ -13335,8 +14128,28 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="CY41">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="CZ41">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DA41">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="DB41">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC41">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="42" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A42" s="9" t="s">
         <v>183</v>
       </c>
@@ -13631,8 +14444,28 @@
         <f t="shared" si="0"/>
         <v>6.6000000000000003E-2</v>
       </c>
+      <c r="CY42">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="CZ42">
+        <f t="shared" si="2"/>
+        <v>0.02</v>
+      </c>
+      <c r="DA42">
+        <f t="shared" si="3"/>
+        <v>0.05</v>
+      </c>
+      <c r="DB42">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC42">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="43" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A43" s="9" t="s">
         <v>184</v>
       </c>
@@ -13923,8 +14756,28 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="CY43">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="CZ43">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DA43">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="DB43">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC43">
+        <f t="shared" si="5"/>
+        <v>0.05</v>
+      </c>
     </row>
-    <row r="44" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A44" s="9" t="s">
         <v>185</v>
       </c>
@@ -14211,8 +15064,28 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="CY44">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="CZ44">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DA44">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="DB44">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC44">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="45" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A45" s="9" t="s">
         <v>143</v>
       </c>
@@ -14499,8 +15372,28 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="CY45">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="CZ45">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DA45">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="DB45">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC45">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="46" spans="1:99" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:107" x14ac:dyDescent="0.3">
       <c r="A46" s="9" t="s">
         <v>186</v>
       </c>
@@ -14787,8 +15680,28 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="CY46">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="CZ46">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DA46">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="DB46">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC46">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="47" spans="1:99" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:107" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A47" s="10" t="s">
         <v>187</v>
       </c>
@@ -15075,8 +15988,28 @@
         <f t="shared" si="0"/>
         <v>7.0519999999999996</v>
       </c>
+      <c r="CY47">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="CZ47">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="DA47">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="DB47">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="DC47">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="48" spans="1:99" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:107" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A48" s="38" t="s">
         <v>66</v>
       </c>
@@ -15337,15 +16270,15 @@
         <v>1</v>
       </c>
       <c r="CJ48" s="58">
-        <f t="shared" ref="CJ48:CL48" si="1">SUM(CJ4:CJ47)</f>
+        <f t="shared" ref="CJ48:CL48" si="6">SUM(CJ4:CJ47)</f>
         <v>1</v>
       </c>
       <c r="CK48" s="58">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>1.0000000000000002</v>
       </c>
       <c r="CL48" s="58">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="CM48" s="58">
@@ -15353,39 +16286,58 @@
         <v>1</v>
       </c>
       <c r="CN48" s="58">
-        <f t="shared" ref="CN48" si="2">SUM(CN4:CN47)</f>
+        <f t="shared" ref="CN48" si="7">SUM(CN4:CN47)</f>
         <v>1</v>
       </c>
       <c r="CO48" s="58">
-        <f t="shared" ref="CO48:CT48" si="3">SUM(CO4:CO47)</f>
+        <f t="shared" ref="CO48:CT48" si="8">SUM(CO4:CO47)</f>
         <v>1</v>
       </c>
       <c r="CP48" s="58">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>1.0000000000000002</v>
       </c>
       <c r="CQ48" s="58">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>1.0000000000000002</v>
       </c>
       <c r="CR48" s="58">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>1.0000000000000002</v>
       </c>
       <c r="CS48" s="58">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="CT48" s="58">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="CU48" s="6">
         <f>SUM(CU3:CU47)</f>
         <v>24.338000000000001</v>
       </c>
+      <c r="CZ48" s="60">
+        <f>SUM(CZ3:CZ47)</f>
+        <v>0.79</v>
+      </c>
+      <c r="DA48" s="60">
+        <f>SUM(DA3:DA47)</f>
+        <v>0.75000000000000022</v>
+      </c>
+      <c r="DB48" s="60">
+        <f t="shared" ref="DB48:DC48" si="9">SUM(DB3:DB47)</f>
+        <v>0.7</v>
+      </c>
+      <c r="DC48" s="60">
+        <f t="shared" si="9"/>
+        <v>0.8</v>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="CY1:DB1"/>
+  </mergeCells>
   <phoneticPr fontId="15" type="noConversion"/>
   <conditionalFormatting sqref="B30:B32">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>

</xml_diff>

<commit_message>
Fix EV and heating network bugs
</commit_message>
<xml_diff>
--- a/districtgenerator/data/SIA2024.xlsx
+++ b/districtgenerator/data/SIA2024.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PycharmProjects\districtgenerator\districtgenerator\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DA02AE6-9A84-4653-AE85-1DECD4D79550}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F42DB278-97FB-469A-A6F3-008B46FBF777}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11835" yWindow="-16335" windowWidth="29040" windowHeight="15720" tabRatio="799" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="799" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SIA2024" sheetId="13" r:id="rId1"/>
@@ -1214,7 +1214,7 @@
       <protection hidden="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
@@ -1280,12 +1280,13 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="18" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="18" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="22">
     <cellStyle name="5x indented GHG Textfiels" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -1598,11 +1599,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:DC48"/>
+  <dimension ref="A1:DC104"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="39.6640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.21875" style="5" customWidth="1"/>
     <col min="3" max="3" width="11.109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.33203125" customWidth="1"/>
@@ -1754,12 +1755,12 @@
       <c r="CH1" s="5" t="s">
         <v>188</v>
       </c>
-      <c r="CY1" s="59" t="s">
+      <c r="CY1" s="60" t="s">
         <v>209</v>
       </c>
-      <c r="CZ1" s="59"/>
-      <c r="DA1" s="59"/>
-      <c r="DB1" s="59"/>
+      <c r="CZ1" s="60"/>
+      <c r="DA1" s="60"/>
+      <c r="DB1" s="60"/>
     </row>
     <row r="2" spans="1:107" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="44" t="s">
@@ -4767,40 +4768,40 @@
         <v>0.1</v>
       </c>
       <c r="BV11" s="16">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="BW11" s="7">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="BX11" s="7">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="BY11" s="7">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="BZ11" s="7">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="CA11" s="7">
         <v>1</v>
       </c>
       <c r="CB11" s="7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CC11" s="7">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="CD11" s="7">
         <v>1</v>
       </c>
       <c r="CE11" s="7">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="CF11" s="7">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="CG11" s="8">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="CH11" s="57">
         <v>0</v>
@@ -5075,40 +5076,40 @@
         <v>0.1</v>
       </c>
       <c r="BV12" s="16">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="BW12" s="7">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="BX12" s="7">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="BY12" s="7">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="BZ12" s="7">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="CA12" s="7">
         <v>1</v>
       </c>
       <c r="CB12" s="7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CC12" s="7">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="CD12" s="7">
         <v>1</v>
       </c>
       <c r="CE12" s="7">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="CF12" s="7">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="CG12" s="8">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="CH12" s="57">
         <v>0</v>
@@ -5383,40 +5384,40 @@
         <v>0.1</v>
       </c>
       <c r="BV13" s="16">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="BW13" s="7">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="BX13" s="7">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="BY13" s="7">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="BZ13" s="7">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="CA13" s="7">
         <v>1</v>
       </c>
       <c r="CB13" s="7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CC13" s="7">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="CD13" s="7">
         <v>1</v>
       </c>
       <c r="CE13" s="7">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="CF13" s="7">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="CG13" s="8">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="CH13" s="57">
         <v>0</v>
@@ -5691,40 +5692,40 @@
         <v>0.1</v>
       </c>
       <c r="BV14" s="16">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="BW14" s="7">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="BX14" s="7">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="BY14" s="7">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="BZ14" s="7">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="CA14" s="7">
         <v>1</v>
       </c>
       <c r="CB14" s="7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CC14" s="7">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="CD14" s="7">
         <v>1</v>
       </c>
       <c r="CE14" s="7">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="CF14" s="7">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="CG14" s="8">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="CH14" s="57">
         <v>0</v>
@@ -16317,22 +16318,806 @@
         <f>SUM(CU3:CU47)</f>
         <v>24.338000000000001</v>
       </c>
-      <c r="CZ48" s="60">
+      <c r="CZ48" s="59">
         <f>SUM(CZ3:CZ47)</f>
         <v>0.79</v>
       </c>
-      <c r="DA48" s="60">
+      <c r="DA48" s="59">
         <f>SUM(DA3:DA47)</f>
         <v>0.75000000000000022</v>
       </c>
-      <c r="DB48" s="60">
+      <c r="DB48" s="59">
         <f t="shared" ref="DB48:DC48" si="9">SUM(DB3:DB47)</f>
         <v>0.7</v>
       </c>
-      <c r="DC48" s="60">
+      <c r="DC48" s="59">
         <f t="shared" si="9"/>
         <v>0.8</v>
       </c>
+    </row>
+    <row r="56" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU56" s="61"/>
+      <c r="BV56" s="61"/>
+      <c r="BW56" s="61"/>
+      <c r="BX56" s="61"/>
+      <c r="BY56" s="61"/>
+      <c r="BZ56" s="61"/>
+      <c r="CA56" s="61"/>
+      <c r="CB56" s="61"/>
+      <c r="CC56" s="61"/>
+      <c r="CD56" s="61"/>
+      <c r="CE56" s="61"/>
+      <c r="CF56" s="61"/>
+      <c r="CG56" s="61"/>
+      <c r="CH56" s="61"/>
+    </row>
+    <row r="57" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU57" s="61"/>
+      <c r="BV57" s="61"/>
+      <c r="BW57" s="61"/>
+      <c r="BX57" s="61"/>
+      <c r="BY57" s="61"/>
+      <c r="BZ57" s="61"/>
+      <c r="CA57" s="61"/>
+      <c r="CB57" s="61"/>
+      <c r="CC57" s="61"/>
+      <c r="CD57" s="61"/>
+      <c r="CE57" s="61"/>
+      <c r="CF57" s="61"/>
+      <c r="CG57" s="61"/>
+      <c r="CH57" s="61"/>
+    </row>
+    <row r="58" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU58" s="61"/>
+      <c r="BV58" s="4"/>
+      <c r="BW58" s="4"/>
+      <c r="BX58" s="4"/>
+      <c r="BY58" s="4"/>
+      <c r="BZ58" s="4"/>
+      <c r="CA58" s="4"/>
+      <c r="CB58" s="4"/>
+      <c r="CC58" s="4"/>
+      <c r="CD58" s="4"/>
+      <c r="CE58" s="4"/>
+      <c r="CF58" s="4"/>
+      <c r="CG58" s="4"/>
+      <c r="CH58" s="61"/>
+    </row>
+    <row r="59" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU59" s="61"/>
+      <c r="BV59" s="4"/>
+      <c r="BW59" s="4"/>
+      <c r="BX59" s="4"/>
+      <c r="BY59" s="4"/>
+      <c r="BZ59" s="4"/>
+      <c r="CA59" s="4"/>
+      <c r="CB59" s="4"/>
+      <c r="CC59" s="4"/>
+      <c r="CD59" s="4"/>
+      <c r="CE59" s="4"/>
+      <c r="CF59" s="4"/>
+      <c r="CG59" s="4"/>
+      <c r="CH59" s="61"/>
+    </row>
+    <row r="60" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU60" s="61"/>
+      <c r="BV60" s="4"/>
+      <c r="BW60" s="4"/>
+      <c r="BX60" s="4"/>
+      <c r="BY60" s="4"/>
+      <c r="BZ60" s="4"/>
+      <c r="CA60" s="4"/>
+      <c r="CB60" s="4"/>
+      <c r="CC60" s="4"/>
+      <c r="CD60" s="4"/>
+      <c r="CE60" s="4"/>
+      <c r="CF60" s="4"/>
+      <c r="CG60" s="4"/>
+      <c r="CH60" s="61"/>
+    </row>
+    <row r="61" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU61" s="61"/>
+      <c r="BV61" s="4"/>
+      <c r="BW61" s="4"/>
+      <c r="BX61" s="4"/>
+      <c r="BY61" s="4"/>
+      <c r="BZ61" s="4"/>
+      <c r="CA61" s="4"/>
+      <c r="CB61" s="4"/>
+      <c r="CC61" s="4"/>
+      <c r="CD61" s="4"/>
+      <c r="CE61" s="4"/>
+      <c r="CF61" s="4"/>
+      <c r="CG61" s="4"/>
+      <c r="CH61" s="61"/>
+    </row>
+    <row r="62" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU62" s="61"/>
+      <c r="BV62" s="4"/>
+      <c r="BW62" s="4"/>
+      <c r="BX62" s="4"/>
+      <c r="BY62" s="4"/>
+      <c r="BZ62" s="4"/>
+      <c r="CA62" s="4"/>
+      <c r="CB62" s="4"/>
+      <c r="CC62" s="4"/>
+      <c r="CD62" s="4"/>
+      <c r="CE62" s="4"/>
+      <c r="CF62" s="4"/>
+      <c r="CG62" s="4"/>
+      <c r="CH62" s="61"/>
+    </row>
+    <row r="63" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU63" s="61"/>
+      <c r="BV63" s="4"/>
+      <c r="BW63" s="4"/>
+      <c r="BX63" s="4"/>
+      <c r="BY63" s="4"/>
+      <c r="BZ63" s="4"/>
+      <c r="CA63" s="4"/>
+      <c r="CB63" s="4"/>
+      <c r="CC63" s="4"/>
+      <c r="CD63" s="4"/>
+      <c r="CE63" s="4"/>
+      <c r="CF63" s="4"/>
+      <c r="CG63" s="4"/>
+      <c r="CH63" s="61"/>
+    </row>
+    <row r="64" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU64" s="61"/>
+      <c r="BV64" s="4"/>
+      <c r="BW64" s="4"/>
+      <c r="BX64" s="4"/>
+      <c r="BY64" s="4"/>
+      <c r="BZ64" s="4"/>
+      <c r="CA64" s="4"/>
+      <c r="CB64" s="4"/>
+      <c r="CC64" s="4"/>
+      <c r="CD64" s="4"/>
+      <c r="CE64" s="4"/>
+      <c r="CF64" s="4"/>
+      <c r="CG64" s="4"/>
+      <c r="CH64" s="61"/>
+    </row>
+    <row r="65" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU65" s="61"/>
+      <c r="BV65" s="4"/>
+      <c r="BW65" s="4"/>
+      <c r="BX65" s="4"/>
+      <c r="BY65" s="4"/>
+      <c r="BZ65" s="4"/>
+      <c r="CA65" s="4"/>
+      <c r="CB65" s="4"/>
+      <c r="CC65" s="4"/>
+      <c r="CD65" s="4"/>
+      <c r="CE65" s="4"/>
+      <c r="CF65" s="4"/>
+      <c r="CG65" s="4"/>
+      <c r="CH65" s="61"/>
+    </row>
+    <row r="66" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU66" s="61"/>
+      <c r="BV66" s="4"/>
+      <c r="BW66" s="4"/>
+      <c r="BX66" s="4"/>
+      <c r="BY66" s="4"/>
+      <c r="BZ66" s="4"/>
+      <c r="CA66" s="4"/>
+      <c r="CB66" s="4"/>
+      <c r="CC66" s="4"/>
+      <c r="CD66" s="4"/>
+      <c r="CE66" s="4"/>
+      <c r="CF66" s="4"/>
+      <c r="CG66" s="4"/>
+      <c r="CH66" s="61"/>
+    </row>
+    <row r="67" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU67" s="61"/>
+      <c r="BV67" s="4"/>
+      <c r="BW67" s="4"/>
+      <c r="BX67" s="4"/>
+      <c r="BY67" s="4"/>
+      <c r="BZ67" s="4"/>
+      <c r="CA67" s="4"/>
+      <c r="CB67" s="4"/>
+      <c r="CC67" s="4"/>
+      <c r="CD67" s="4"/>
+      <c r="CE67" s="4"/>
+      <c r="CF67" s="4"/>
+      <c r="CG67" s="4"/>
+      <c r="CH67" s="61"/>
+    </row>
+    <row r="68" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU68" s="61"/>
+      <c r="BV68" s="4"/>
+      <c r="BW68" s="4"/>
+      <c r="BX68" s="4"/>
+      <c r="BY68" s="4"/>
+      <c r="BZ68" s="4"/>
+      <c r="CA68" s="4"/>
+      <c r="CB68" s="4"/>
+      <c r="CC68" s="4"/>
+      <c r="CD68" s="4"/>
+      <c r="CE68" s="4"/>
+      <c r="CF68" s="4"/>
+      <c r="CG68" s="4"/>
+      <c r="CH68" s="61"/>
+    </row>
+    <row r="69" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU69" s="61"/>
+      <c r="BV69" s="4"/>
+      <c r="BW69" s="4"/>
+      <c r="BX69" s="4"/>
+      <c r="BY69" s="4"/>
+      <c r="BZ69" s="4"/>
+      <c r="CA69" s="4"/>
+      <c r="CB69" s="4"/>
+      <c r="CC69" s="4"/>
+      <c r="CD69" s="4"/>
+      <c r="CE69" s="4"/>
+      <c r="CF69" s="4"/>
+      <c r="CG69" s="4"/>
+      <c r="CH69" s="61"/>
+    </row>
+    <row r="70" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU70" s="61"/>
+      <c r="BV70" s="4"/>
+      <c r="BW70" s="4"/>
+      <c r="BX70" s="4"/>
+      <c r="BY70" s="4"/>
+      <c r="BZ70" s="4"/>
+      <c r="CA70" s="4"/>
+      <c r="CB70" s="4"/>
+      <c r="CC70" s="4"/>
+      <c r="CD70" s="4"/>
+      <c r="CE70" s="4"/>
+      <c r="CF70" s="4"/>
+      <c r="CG70" s="4"/>
+      <c r="CH70" s="61"/>
+    </row>
+    <row r="71" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU71" s="61"/>
+      <c r="BV71" s="4"/>
+      <c r="BW71" s="4"/>
+      <c r="BX71" s="4"/>
+      <c r="BY71" s="4"/>
+      <c r="BZ71" s="4"/>
+      <c r="CA71" s="4"/>
+      <c r="CB71" s="4"/>
+      <c r="CC71" s="4"/>
+      <c r="CD71" s="4"/>
+      <c r="CE71" s="4"/>
+      <c r="CF71" s="4"/>
+      <c r="CG71" s="4"/>
+      <c r="CH71" s="61"/>
+    </row>
+    <row r="72" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU72" s="61"/>
+      <c r="BV72" s="4"/>
+      <c r="BW72" s="4"/>
+      <c r="BX72" s="4"/>
+      <c r="BY72" s="4"/>
+      <c r="BZ72" s="4"/>
+      <c r="CA72" s="4"/>
+      <c r="CB72" s="4"/>
+      <c r="CC72" s="4"/>
+      <c r="CD72" s="4"/>
+      <c r="CE72" s="4"/>
+      <c r="CF72" s="4"/>
+      <c r="CG72" s="4"/>
+      <c r="CH72" s="61"/>
+    </row>
+    <row r="73" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU73" s="61"/>
+      <c r="BV73" s="4"/>
+      <c r="BW73" s="4"/>
+      <c r="BX73" s="4"/>
+      <c r="BY73" s="4"/>
+      <c r="BZ73" s="4"/>
+      <c r="CA73" s="4"/>
+      <c r="CB73" s="4"/>
+      <c r="CC73" s="4"/>
+      <c r="CD73" s="4"/>
+      <c r="CE73" s="4"/>
+      <c r="CF73" s="4"/>
+      <c r="CG73" s="4"/>
+      <c r="CH73" s="61"/>
+    </row>
+    <row r="74" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU74" s="61"/>
+      <c r="BV74" s="4"/>
+      <c r="BW74" s="4"/>
+      <c r="BX74" s="4"/>
+      <c r="BY74" s="4"/>
+      <c r="BZ74" s="4"/>
+      <c r="CA74" s="4"/>
+      <c r="CB74" s="4"/>
+      <c r="CC74" s="4"/>
+      <c r="CD74" s="4"/>
+      <c r="CE74" s="4"/>
+      <c r="CF74" s="4"/>
+      <c r="CG74" s="4"/>
+      <c r="CH74" s="61"/>
+    </row>
+    <row r="75" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU75" s="61"/>
+      <c r="BV75" s="4"/>
+      <c r="BW75" s="4"/>
+      <c r="BX75" s="4"/>
+      <c r="BY75" s="4"/>
+      <c r="BZ75" s="4"/>
+      <c r="CA75" s="4"/>
+      <c r="CB75" s="4"/>
+      <c r="CC75" s="4"/>
+      <c r="CD75" s="4"/>
+      <c r="CE75" s="4"/>
+      <c r="CF75" s="4"/>
+      <c r="CG75" s="4"/>
+      <c r="CH75" s="61"/>
+    </row>
+    <row r="76" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU76" s="61"/>
+      <c r="BV76" s="4"/>
+      <c r="BW76" s="4"/>
+      <c r="BX76" s="4"/>
+      <c r="BY76" s="4"/>
+      <c r="BZ76" s="4"/>
+      <c r="CA76" s="4"/>
+      <c r="CB76" s="4"/>
+      <c r="CC76" s="4"/>
+      <c r="CD76" s="4"/>
+      <c r="CE76" s="4"/>
+      <c r="CF76" s="4"/>
+      <c r="CG76" s="4"/>
+      <c r="CH76" s="61"/>
+    </row>
+    <row r="77" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU77" s="61"/>
+      <c r="BV77" s="4"/>
+      <c r="BW77" s="4"/>
+      <c r="BX77" s="4"/>
+      <c r="BY77" s="4"/>
+      <c r="BZ77" s="4"/>
+      <c r="CA77" s="4"/>
+      <c r="CB77" s="4"/>
+      <c r="CC77" s="4"/>
+      <c r="CD77" s="4"/>
+      <c r="CE77" s="4"/>
+      <c r="CF77" s="4"/>
+      <c r="CG77" s="4"/>
+      <c r="CH77" s="61"/>
+    </row>
+    <row r="78" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU78" s="61"/>
+      <c r="BV78" s="4"/>
+      <c r="BW78" s="4"/>
+      <c r="BX78" s="4"/>
+      <c r="BY78" s="4"/>
+      <c r="BZ78" s="4"/>
+      <c r="CA78" s="4"/>
+      <c r="CB78" s="4"/>
+      <c r="CC78" s="4"/>
+      <c r="CD78" s="4"/>
+      <c r="CE78" s="4"/>
+      <c r="CF78" s="4"/>
+      <c r="CG78" s="4"/>
+      <c r="CH78" s="61"/>
+    </row>
+    <row r="79" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU79" s="61"/>
+      <c r="BV79" s="4"/>
+      <c r="BW79" s="4"/>
+      <c r="BX79" s="4"/>
+      <c r="BY79" s="4"/>
+      <c r="BZ79" s="4"/>
+      <c r="CA79" s="4"/>
+      <c r="CB79" s="4"/>
+      <c r="CC79" s="4"/>
+      <c r="CD79" s="4"/>
+      <c r="CE79" s="4"/>
+      <c r="CF79" s="4"/>
+      <c r="CG79" s="4"/>
+      <c r="CH79" s="61"/>
+    </row>
+    <row r="80" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU80" s="61"/>
+      <c r="BV80" s="4"/>
+      <c r="BW80" s="4"/>
+      <c r="BX80" s="4"/>
+      <c r="BY80" s="4"/>
+      <c r="BZ80" s="4"/>
+      <c r="CA80" s="4"/>
+      <c r="CB80" s="4"/>
+      <c r="CC80" s="4"/>
+      <c r="CD80" s="4"/>
+      <c r="CE80" s="4"/>
+      <c r="CF80" s="4"/>
+      <c r="CG80" s="4"/>
+      <c r="CH80" s="61"/>
+    </row>
+    <row r="81" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU81" s="61"/>
+      <c r="BV81" s="4"/>
+      <c r="BW81" s="4"/>
+      <c r="BX81" s="4"/>
+      <c r="BY81" s="4"/>
+      <c r="BZ81" s="4"/>
+      <c r="CA81" s="4"/>
+      <c r="CB81" s="4"/>
+      <c r="CC81" s="4"/>
+      <c r="CD81" s="4"/>
+      <c r="CE81" s="4"/>
+      <c r="CF81" s="4"/>
+      <c r="CG81" s="4"/>
+      <c r="CH81" s="61"/>
+    </row>
+    <row r="82" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU82" s="61"/>
+      <c r="BV82" s="4"/>
+      <c r="BW82" s="4"/>
+      <c r="BX82" s="4"/>
+      <c r="BY82" s="4"/>
+      <c r="BZ82" s="4"/>
+      <c r="CA82" s="4"/>
+      <c r="CB82" s="4"/>
+      <c r="CC82" s="4"/>
+      <c r="CD82" s="4"/>
+      <c r="CE82" s="4"/>
+      <c r="CF82" s="4"/>
+      <c r="CG82" s="4"/>
+      <c r="CH82" s="61"/>
+    </row>
+    <row r="83" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU83" s="61"/>
+      <c r="BV83" s="4"/>
+      <c r="BW83" s="4"/>
+      <c r="BX83" s="4"/>
+      <c r="BY83" s="4"/>
+      <c r="BZ83" s="4"/>
+      <c r="CA83" s="4"/>
+      <c r="CB83" s="4"/>
+      <c r="CC83" s="4"/>
+      <c r="CD83" s="4"/>
+      <c r="CE83" s="4"/>
+      <c r="CF83" s="4"/>
+      <c r="CG83" s="4"/>
+      <c r="CH83" s="61"/>
+    </row>
+    <row r="84" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU84" s="61"/>
+      <c r="BV84" s="4"/>
+      <c r="BW84" s="4"/>
+      <c r="BX84" s="4"/>
+      <c r="BY84" s="4"/>
+      <c r="BZ84" s="4"/>
+      <c r="CA84" s="4"/>
+      <c r="CB84" s="4"/>
+      <c r="CC84" s="4"/>
+      <c r="CD84" s="4"/>
+      <c r="CE84" s="4"/>
+      <c r="CF84" s="4"/>
+      <c r="CG84" s="4"/>
+      <c r="CH84" s="61"/>
+    </row>
+    <row r="85" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU85" s="61"/>
+      <c r="BV85" s="4"/>
+      <c r="BW85" s="4"/>
+      <c r="BX85" s="4"/>
+      <c r="BY85" s="4"/>
+      <c r="BZ85" s="4"/>
+      <c r="CA85" s="4"/>
+      <c r="CB85" s="4"/>
+      <c r="CC85" s="4"/>
+      <c r="CD85" s="4"/>
+      <c r="CE85" s="4"/>
+      <c r="CF85" s="4"/>
+      <c r="CG85" s="4"/>
+      <c r="CH85" s="61"/>
+    </row>
+    <row r="86" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU86" s="61"/>
+      <c r="BV86" s="4"/>
+      <c r="BW86" s="4"/>
+      <c r="BX86" s="4"/>
+      <c r="BY86" s="4"/>
+      <c r="BZ86" s="4"/>
+      <c r="CA86" s="4"/>
+      <c r="CB86" s="4"/>
+      <c r="CC86" s="4"/>
+      <c r="CD86" s="4"/>
+      <c r="CE86" s="4"/>
+      <c r="CF86" s="4"/>
+      <c r="CG86" s="4"/>
+      <c r="CH86" s="61"/>
+    </row>
+    <row r="87" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU87" s="61"/>
+      <c r="BV87" s="4"/>
+      <c r="BW87" s="4"/>
+      <c r="BX87" s="4"/>
+      <c r="BY87" s="4"/>
+      <c r="BZ87" s="4"/>
+      <c r="CA87" s="4"/>
+      <c r="CB87" s="4"/>
+      <c r="CC87" s="4"/>
+      <c r="CD87" s="4"/>
+      <c r="CE87" s="4"/>
+      <c r="CF87" s="4"/>
+      <c r="CG87" s="4"/>
+      <c r="CH87" s="61"/>
+    </row>
+    <row r="88" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU88" s="61"/>
+      <c r="BV88" s="4"/>
+      <c r="BW88" s="4"/>
+      <c r="BX88" s="4"/>
+      <c r="BY88" s="4"/>
+      <c r="BZ88" s="4"/>
+      <c r="CA88" s="4"/>
+      <c r="CB88" s="4"/>
+      <c r="CC88" s="4"/>
+      <c r="CD88" s="4"/>
+      <c r="CE88" s="4"/>
+      <c r="CF88" s="4"/>
+      <c r="CG88" s="4"/>
+      <c r="CH88" s="61"/>
+    </row>
+    <row r="89" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU89" s="61"/>
+      <c r="BV89" s="4"/>
+      <c r="BW89" s="4"/>
+      <c r="BX89" s="4"/>
+      <c r="BY89" s="4"/>
+      <c r="BZ89" s="4"/>
+      <c r="CA89" s="4"/>
+      <c r="CB89" s="4"/>
+      <c r="CC89" s="4"/>
+      <c r="CD89" s="4"/>
+      <c r="CE89" s="4"/>
+      <c r="CF89" s="4"/>
+      <c r="CG89" s="4"/>
+      <c r="CH89" s="61"/>
+    </row>
+    <row r="90" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU90" s="61"/>
+      <c r="BV90" s="4"/>
+      <c r="BW90" s="4"/>
+      <c r="BX90" s="4"/>
+      <c r="BY90" s="4"/>
+      <c r="BZ90" s="4"/>
+      <c r="CA90" s="4"/>
+      <c r="CB90" s="4"/>
+      <c r="CC90" s="4"/>
+      <c r="CD90" s="4"/>
+      <c r="CE90" s="4"/>
+      <c r="CF90" s="4"/>
+      <c r="CG90" s="4"/>
+      <c r="CH90" s="61"/>
+    </row>
+    <row r="91" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU91" s="61"/>
+      <c r="BV91" s="4"/>
+      <c r="BW91" s="4"/>
+      <c r="BX91" s="4"/>
+      <c r="BY91" s="4"/>
+      <c r="BZ91" s="4"/>
+      <c r="CA91" s="4"/>
+      <c r="CB91" s="4"/>
+      <c r="CC91" s="4"/>
+      <c r="CD91" s="4"/>
+      <c r="CE91" s="4"/>
+      <c r="CF91" s="4"/>
+      <c r="CG91" s="4"/>
+      <c r="CH91" s="61"/>
+    </row>
+    <row r="92" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU92" s="61"/>
+      <c r="BV92" s="4"/>
+      <c r="BW92" s="4"/>
+      <c r="BX92" s="4"/>
+      <c r="BY92" s="4"/>
+      <c r="BZ92" s="4"/>
+      <c r="CA92" s="4"/>
+      <c r="CB92" s="4"/>
+      <c r="CC92" s="4"/>
+      <c r="CD92" s="4"/>
+      <c r="CE92" s="4"/>
+      <c r="CF92" s="4"/>
+      <c r="CG92" s="4"/>
+      <c r="CH92" s="61"/>
+    </row>
+    <row r="93" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU93" s="61"/>
+      <c r="BV93" s="4"/>
+      <c r="BW93" s="4"/>
+      <c r="BX93" s="4"/>
+      <c r="BY93" s="4"/>
+      <c r="BZ93" s="4"/>
+      <c r="CA93" s="4"/>
+      <c r="CB93" s="4"/>
+      <c r="CC93" s="4"/>
+      <c r="CD93" s="4"/>
+      <c r="CE93" s="4"/>
+      <c r="CF93" s="4"/>
+      <c r="CG93" s="4"/>
+      <c r="CH93" s="61"/>
+    </row>
+    <row r="94" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU94" s="61"/>
+      <c r="BV94" s="4"/>
+      <c r="BW94" s="4"/>
+      <c r="BX94" s="4"/>
+      <c r="BY94" s="4"/>
+      <c r="BZ94" s="4"/>
+      <c r="CA94" s="4"/>
+      <c r="CB94" s="4"/>
+      <c r="CC94" s="4"/>
+      <c r="CD94" s="4"/>
+      <c r="CE94" s="4"/>
+      <c r="CF94" s="4"/>
+      <c r="CG94" s="4"/>
+      <c r="CH94" s="61"/>
+    </row>
+    <row r="95" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU95" s="61"/>
+      <c r="BV95" s="4"/>
+      <c r="BW95" s="4"/>
+      <c r="BX95" s="4"/>
+      <c r="BY95" s="4"/>
+      <c r="BZ95" s="4"/>
+      <c r="CA95" s="4"/>
+      <c r="CB95" s="4"/>
+      <c r="CC95" s="4"/>
+      <c r="CD95" s="4"/>
+      <c r="CE95" s="4"/>
+      <c r="CF95" s="4"/>
+      <c r="CG95" s="4"/>
+      <c r="CH95" s="61"/>
+    </row>
+    <row r="96" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU96" s="61"/>
+      <c r="BV96" s="4"/>
+      <c r="BW96" s="4"/>
+      <c r="BX96" s="4"/>
+      <c r="BY96" s="4"/>
+      <c r="BZ96" s="4"/>
+      <c r="CA96" s="4"/>
+      <c r="CB96" s="4"/>
+      <c r="CC96" s="4"/>
+      <c r="CD96" s="4"/>
+      <c r="CE96" s="4"/>
+      <c r="CF96" s="4"/>
+      <c r="CG96" s="4"/>
+      <c r="CH96" s="61"/>
+    </row>
+    <row r="97" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU97" s="61"/>
+      <c r="BV97" s="4"/>
+      <c r="BW97" s="4"/>
+      <c r="BX97" s="4"/>
+      <c r="BY97" s="4"/>
+      <c r="BZ97" s="4"/>
+      <c r="CA97" s="4"/>
+      <c r="CB97" s="4"/>
+      <c r="CC97" s="4"/>
+      <c r="CD97" s="4"/>
+      <c r="CE97" s="4"/>
+      <c r="CF97" s="4"/>
+      <c r="CG97" s="4"/>
+      <c r="CH97" s="61"/>
+    </row>
+    <row r="98" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU98" s="61"/>
+      <c r="BV98" s="4"/>
+      <c r="BW98" s="4"/>
+      <c r="BX98" s="4"/>
+      <c r="BY98" s="4"/>
+      <c r="BZ98" s="4"/>
+      <c r="CA98" s="4"/>
+      <c r="CB98" s="4"/>
+      <c r="CC98" s="4"/>
+      <c r="CD98" s="4"/>
+      <c r="CE98" s="4"/>
+      <c r="CF98" s="4"/>
+      <c r="CG98" s="4"/>
+      <c r="CH98" s="61"/>
+    </row>
+    <row r="99" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU99" s="61"/>
+      <c r="BV99" s="4"/>
+      <c r="BW99" s="4"/>
+      <c r="BX99" s="4"/>
+      <c r="BY99" s="4"/>
+      <c r="BZ99" s="4"/>
+      <c r="CA99" s="4"/>
+      <c r="CB99" s="4"/>
+      <c r="CC99" s="4"/>
+      <c r="CD99" s="4"/>
+      <c r="CE99" s="4"/>
+      <c r="CF99" s="4"/>
+      <c r="CG99" s="4"/>
+      <c r="CH99" s="61"/>
+    </row>
+    <row r="100" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU100" s="61"/>
+      <c r="BV100" s="4"/>
+      <c r="BW100" s="4"/>
+      <c r="BX100" s="4"/>
+      <c r="BY100" s="4"/>
+      <c r="BZ100" s="4"/>
+      <c r="CA100" s="4"/>
+      <c r="CB100" s="4"/>
+      <c r="CC100" s="4"/>
+      <c r="CD100" s="4"/>
+      <c r="CE100" s="4"/>
+      <c r="CF100" s="4"/>
+      <c r="CG100" s="4"/>
+      <c r="CH100" s="61"/>
+    </row>
+    <row r="101" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU101" s="61"/>
+      <c r="BV101" s="4"/>
+      <c r="BW101" s="4"/>
+      <c r="BX101" s="4"/>
+      <c r="BY101" s="4"/>
+      <c r="BZ101" s="4"/>
+      <c r="CA101" s="4"/>
+      <c r="CB101" s="4"/>
+      <c r="CC101" s="4"/>
+      <c r="CD101" s="4"/>
+      <c r="CE101" s="4"/>
+      <c r="CF101" s="4"/>
+      <c r="CG101" s="4"/>
+      <c r="CH101" s="61"/>
+    </row>
+    <row r="102" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU102" s="61"/>
+      <c r="BV102" s="4"/>
+      <c r="BW102" s="4"/>
+      <c r="BX102" s="4"/>
+      <c r="BY102" s="4"/>
+      <c r="BZ102" s="4"/>
+      <c r="CA102" s="4"/>
+      <c r="CB102" s="4"/>
+      <c r="CC102" s="4"/>
+      <c r="CD102" s="4"/>
+      <c r="CE102" s="4"/>
+      <c r="CF102" s="4"/>
+      <c r="CG102" s="4"/>
+      <c r="CH102" s="61"/>
+    </row>
+    <row r="103" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU103" s="61"/>
+      <c r="BV103" s="61"/>
+      <c r="BW103" s="61"/>
+      <c r="BX103" s="61"/>
+      <c r="BY103" s="61"/>
+      <c r="BZ103" s="61"/>
+      <c r="CA103" s="61"/>
+      <c r="CB103" s="61"/>
+      <c r="CC103" s="61"/>
+      <c r="CD103" s="61"/>
+      <c r="CE103" s="61"/>
+      <c r="CF103" s="61"/>
+      <c r="CG103" s="61"/>
+      <c r="CH103" s="61"/>
+    </row>
+    <row r="104" spans="73:86" x14ac:dyDescent="0.3">
+      <c r="BU104" s="61"/>
+      <c r="BV104" s="61"/>
+      <c r="BW104" s="61"/>
+      <c r="BX104" s="61"/>
+      <c r="BY104" s="61"/>
+      <c r="BZ104" s="61"/>
+      <c r="CA104" s="61"/>
+      <c r="CB104" s="61"/>
+      <c r="CC104" s="61"/>
+      <c r="CD104" s="61"/>
+      <c r="CE104" s="61"/>
+      <c r="CF104" s="61"/>
+      <c r="CG104" s="61"/>
+      <c r="CH104" s="61"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>